<commit_message>
Fix: Correct Open Finance coverage - only 39 localized, 13 Solo Skandia
</commit_message>
<xml_diff>
--- a/Open_Finance_Datos_Simulados.xlsx
+++ b/Open_Finance_Datos_Simulados.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -509,27 +509,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1090825067</t>
+          <t>1090000111</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Maria Fernanda Cardenas Suarez</t>
+          <t>Silvia Gutierrez</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>maria.fernanda32_backup@correo.com</t>
+          <t>silvia.gutierrez76_backup@correo.com</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7748301</v>
+        <v>1996853</v>
       </c>
       <c r="E2" t="n">
-        <v>5378300</v>
+        <v>5236215</v>
       </c>
       <c r="F2" t="n">
-        <v>508</v>
+        <v>396</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -538,7 +538,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Fondo de inversion, Pension voluntaria, Cesantias</t>
+          <t>Seguro de vida, Fondo de inversion, Cesantias</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -547,39 +547,39 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>2301785</v>
+        <v>2622820</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>46205.56031574074</v>
+        <v>46258.56031574074</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>900000002-0</t>
+          <t>1090000112</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Agroindustrias del Norte S.A.S.</t>
+          <t>Diego Sanchez</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>agroindustrias.del29_backup@correo.com</t>
+          <t>diego.sanchez74@example.com</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7427508</v>
+        <v>1849382</v>
       </c>
       <c r="E3" t="n">
-        <v>5772837</v>
+        <v>2931991</v>
       </c>
       <c r="F3" t="n">
-        <v>480</v>
+        <v>307</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -588,48 +588,48 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Seguro de vida, Cesantias, Pension obligatoria</t>
+          <t>Pension voluntaria</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ACTIVA</t>
+          <t>SUSPENDIDA</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>691572</v>
+        <v>3686220</v>
       </c>
       <c r="K3" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>46219.56031574074</v>
+        <v>46214.56031574074</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1090000100</t>
+          <t>1090000113</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Andres Cruz</t>
+          <t>Patricia Vargas</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>andres.26@outlook.com</t>
+          <t>patricia.vargas98@example.com</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6150180</v>
+        <v>1592188</v>
       </c>
       <c r="E4" t="n">
-        <v>5769896</v>
+        <v>2955533</v>
       </c>
       <c r="F4" t="n">
-        <v>766</v>
+        <v>448</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -638,7 +638,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Fondo de inversion, Pension voluntaria</t>
+          <t>Pension obligatoria, Pension voluntaria, Fondo de inversion</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -647,48 +647,48 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2433685</v>
+        <v>166543</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>46190.56031574074</v>
+        <v>46266.56031574074</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1090000101</t>
+          <t>1090000114</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mariana Hernandez</t>
+          <t>Carlos Rodriguez</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>mariana.hernandez22_backup@correo.com</t>
+          <t>carlos.rodriguez54_backup@correo.com</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>9533862</v>
+        <v>4701831</v>
       </c>
       <c r="E5" t="n">
-        <v>2909538</v>
+        <v>2565150</v>
       </c>
       <c r="F5" t="n">
-        <v>784</v>
+        <v>758</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Pension obligatoria</t>
+          <t>Seguro de vida, Fondo de inversion, Pension voluntaria</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -697,48 +697,48 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>3125495</v>
+        <v>4954215</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>46234.56031574074</v>
+        <v>46195.56031574074</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1090000102</t>
+          <t>1090000115</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rosa Ramirez</t>
+          <t>Fernando Lopez</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>rosa.ramirez30_backup@correo.com</t>
+          <t>fernando.lopez84@example.com</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4124464</v>
+        <v>2636917</v>
       </c>
       <c r="E6" t="n">
-        <v>3626606</v>
+        <v>1617707</v>
       </c>
       <c r="F6" t="n">
-        <v>466</v>
+        <v>499</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Seguro de vida, Pension voluntaria</t>
+          <t>Fondo de inversion, Cesantias</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -747,39 +747,39 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>2901943</v>
+        <v>2125844</v>
       </c>
       <c r="K6" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>46237.56031574074</v>
+        <v>46265.56031574074</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1090000103</t>
+          <t>1090000116</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Roberto Cruz</t>
+          <t>Silvia Torres</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>roberto.cruz8_backup@correo.com</t>
+          <t>silvia.torres41_backup@correo.com</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4703444</v>
+        <v>3467171</v>
       </c>
       <c r="E7" t="n">
-        <v>4903224</v>
+        <v>2064394</v>
       </c>
       <c r="F7" t="n">
-        <v>595</v>
+        <v>310</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -788,7 +788,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Fondo de inversion, Seguro de vida</t>
+          <t>Cesantias, Fondo de inversion, Pension obligatoria</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -797,48 +797,48 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1599596</v>
+        <v>4809958</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>46253.56031574074</v>
+        <v>46252.56031574074</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1090000104</t>
+          <t>1090000117</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Diego Vargas</t>
+          <t>Silvia Torres</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>diego.vargas7_backup@correo.com</t>
+          <t>silvia.torres25_backup@correo.com</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>7820299</v>
+        <v>9290799</v>
       </c>
       <c r="E8" t="n">
-        <v>3791351</v>
+        <v>4509895</v>
       </c>
       <c r="F8" t="n">
-        <v>600</v>
+        <v>573</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Cesantias, Pension voluntaria</t>
+          <t>Fondo de inversion, Seguro de vida, Pension voluntaria</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -847,48 +847,48 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1491290</v>
+        <v>2496870</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>46267.56031574074</v>
+        <v>46223.56031574074</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1090000105</t>
+          <t>1090000118</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Patricia Moreno</t>
+          <t>Fernando Rodriguez</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>patricia.moreno70_backup@correo.com</t>
+          <t>fernando.rodriguez9@example.com</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2843294</v>
+        <v>9261337</v>
       </c>
       <c r="E9" t="n">
-        <v>3912094</v>
+        <v>5191025</v>
       </c>
       <c r="F9" t="n">
-        <v>416</v>
+        <v>733</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Pension voluntaria, Seguro de vida, Cesantias</t>
+          <t>Fondo de inversion</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -897,39 +897,39 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>2266327</v>
+        <v>2800959</v>
       </c>
       <c r="K9" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>46228.56031574074</v>
+        <v>46187.56031574074</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1090000106</t>
+          <t>1090000119</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mariana Castillo</t>
+          <t>Juan Castillo</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>mariana.17@empresa.com.co</t>
+          <t>juan.84@gmail.com</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4795743</v>
+        <v>7049002</v>
       </c>
       <c r="E10" t="n">
-        <v>5868677</v>
+        <v>1122053</v>
       </c>
       <c r="F10" t="n">
-        <v>326</v>
+        <v>497</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Pension obligatoria, Cesantias, Seguro de vida</t>
+          <t>Pension obligatoria</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -947,48 +947,48 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>4723361</v>
+        <v>4535581</v>
       </c>
       <c r="K10" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>46242.56031574074</v>
+        <v>46191.56031574074</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1090000107</t>
+          <t>1090000120</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Andres Martinez</t>
+          <t>Diego Sanchez</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>andres.martinez20_backup@correo.com</t>
+          <t>diego.sanchez51_backup@correo.com</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3869515</v>
+        <v>8297927</v>
       </c>
       <c r="E11" t="n">
-        <v>2626582</v>
+        <v>3839880</v>
       </c>
       <c r="F11" t="n">
-        <v>377</v>
+        <v>338</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Pension obligatoria, Pension voluntaria, Cesantias</t>
+          <t>Fondo de inversion, Pension obligatoria</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -997,39 +997,39 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>3225622</v>
+        <v>4211538</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>46241.56031574074</v>
+        <v>46203.56031575231</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1090000108</t>
+          <t>1090000121</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fernando Gutierrez</t>
+          <t>Roberto Dominguez</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>fernando.gutierrez57_backup@correo.com</t>
+          <t>roberto.dominguez18_backup@correo.com</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>9009643</v>
+        <v>8627814</v>
       </c>
       <c r="E12" t="n">
-        <v>5929704</v>
+        <v>2530938</v>
       </c>
       <c r="F12" t="n">
-        <v>450</v>
+        <v>770</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Pension voluntaria</t>
+          <t>Pension voluntaria, Pension obligatoria</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,39 +1047,39 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>327690</v>
+        <v>238829</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>46240.56031574074</v>
+        <v>46269.56031575231</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1090000109</t>
+          <t>1090000122</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Maria Vargas</t>
+          <t>Andres Hernandez</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>maria.vargas65_backup@correo.com</t>
+          <t>andres.hernandez79_backup@correo.com</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>8101605</v>
+        <v>7852221</v>
       </c>
       <c r="E13" t="n">
-        <v>3560269</v>
+        <v>4043319</v>
       </c>
       <c r="F13" t="n">
-        <v>656</v>
+        <v>503</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Cesantias, Fondo de inversion</t>
+          <t>Pension voluntaria, Seguro de vida</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1097,69 +1097,69 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>3871268</v>
+        <v>2447891</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>46195.56031574074</v>
+        <v>46192.56031575231</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1090000110</t>
+          <t>1090000123</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Silvia Torres</t>
+          <t>Fernando Lopez</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>silvia.torres33_backup@correo.com</t>
+          <t>fernando.lopez77_backup@correo.com</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>9940045</v>
+        <v>7551769</v>
       </c>
       <c r="E14" t="n">
-        <v>2827142</v>
+        <v>3702630</v>
       </c>
       <c r="F14" t="n">
-        <v>749</v>
+        <v>769</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Pension obligatoria, Pension voluntaria, Cesantias</t>
+          <t>Seguro de vida, Pension voluntaria</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ACTIVA</t>
+          <t>SUSPENDIDA</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>2428679</v>
+        <v>3349132</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>46201.56031574074</v>
+        <v>46226.56031575231</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1090000111</t>
+          <t>1090000124</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1169,26 +1169,26 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>silvia.gutierrez76_backup@correo.com</t>
+          <t>silvia.87@outlook.com</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1996853</v>
+        <v>3950157</v>
       </c>
       <c r="E15" t="n">
-        <v>5236215</v>
+        <v>3230906</v>
       </c>
       <c r="F15" t="n">
-        <v>396</v>
+        <v>826</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Seguro de vida, Fondo de inversion, Cesantias</t>
+          <t>Pension obligatoria, Cesantias</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1197,39 +1197,39 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>2622820</v>
+        <v>3010491</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>46258.56031574074</v>
+        <v>46216.56031575231</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1090000112</t>
+          <t>1090000125</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Diego Sanchez</t>
+          <t>Ana Vargas</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>diego.sanchez74@example.com</t>
+          <t>ana.vargas93_backup@correo.com</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1849382</v>
+        <v>4762974</v>
       </c>
       <c r="E16" t="n">
-        <v>2931991</v>
+        <v>5360377</v>
       </c>
       <c r="F16" t="n">
-        <v>307</v>
+        <v>330</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Pension voluntaria</t>
+          <t>Pension obligatoria</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1247,39 +1247,39 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>3686220</v>
+        <v>1208058</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>46214.56031574074</v>
+        <v>46186.56031575231</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1090000113</t>
+          <t>1090000126</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Patricia Vargas</t>
+          <t>Sandra Ramirez</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>patricia.vargas98@example.com</t>
+          <t>sandra.82@outlook.com</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1592188</v>
+        <v>5139802</v>
       </c>
       <c r="E17" t="n">
-        <v>2955533</v>
+        <v>1606064</v>
       </c>
       <c r="F17" t="n">
-        <v>448</v>
+        <v>688</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Pension obligatoria, Pension voluntaria, Fondo de inversion</t>
+          <t>Pension voluntaria, Fondo de inversion</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1297,48 +1297,48 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>166543</v>
+        <v>697999</v>
       </c>
       <c r="K17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>46266.56031574074</v>
+        <v>46241.56031575231</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1090000114</t>
+          <t>1090000127</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Carlos Rodriguez</t>
+          <t>Miguel Cruz</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>carlos.rodriguez54_backup@correo.com</t>
+          <t>miguel.42@empresa.com.co</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4701831</v>
+        <v>2931284</v>
       </c>
       <c r="E18" t="n">
-        <v>2565150</v>
+        <v>2864732</v>
       </c>
       <c r="F18" t="n">
-        <v>758</v>
+        <v>463</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Seguro de vida, Fondo de inversion, Pension voluntaria</t>
+          <t>Pension voluntaria</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1347,39 +1347,39 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>4954215</v>
+        <v>2382433</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>46195.56031574074</v>
+        <v>46263.56031575231</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1090000115</t>
+          <t>1090000128</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Fernando Lopez</t>
+          <t>Juan Rodriguez</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>fernando.lopez84@example.com</t>
+          <t>juan.rodriguez62@example.com</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2636917</v>
+        <v>5710501</v>
       </c>
       <c r="E19" t="n">
-        <v>1617707</v>
+        <v>3014887</v>
       </c>
       <c r="F19" t="n">
-        <v>499</v>
+        <v>796</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1388,48 +1388,48 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Fondo de inversion, Cesantias</t>
+          <t>Fondo de inversion, Pension obligatoria</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>ACTIVA</t>
+          <t>SUSPENDIDA</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>2125844</v>
+        <v>2570265</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>46265.56031574074</v>
+        <v>46235.56031575231</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1090000116</t>
+          <t>1090000129</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Silvia Torres</t>
+          <t>Fernando Dominguez</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>silvia.torres41_backup@correo.com</t>
+          <t>fernando.dominguez3_backup@correo.com</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3467171</v>
+        <v>9100219</v>
       </c>
       <c r="E20" t="n">
-        <v>2064394</v>
+        <v>4123750</v>
       </c>
       <c r="F20" t="n">
-        <v>310</v>
+        <v>422</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Cesantias, Fondo de inversion, Pension obligatoria</t>
+          <t>Cesantias</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1447,39 +1447,39 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>4809958</v>
+        <v>4226540</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>46252.56031574074</v>
+        <v>46249.56031575231</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1090000117</t>
+          <t>1090000130</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Silvia Torres</t>
+          <t>Diego Martinez</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>silvia.torres25_backup@correo.com</t>
+          <t>diego.martinez74@example.com</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>9290799</v>
+        <v>7343863</v>
       </c>
       <c r="E21" t="n">
-        <v>4509895</v>
+        <v>4172992</v>
       </c>
       <c r="F21" t="n">
-        <v>573</v>
+        <v>380</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1488,28 +1488,28 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Fondo de inversion, Seguro de vida, Pension voluntaria</t>
+          <t>Pension obligatoria, Pension voluntaria, Cesantias</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>ACTIVA</t>
+          <t>SUSPENDIDA</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>2496870</v>
+        <v>192832</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>46223.56031574074</v>
+        <v>46246.56031575231</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1090000118</t>
+          <t>1090000131</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1519,17 +1519,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>fernando.rodriguez9@example.com</t>
+          <t>fernando.rodriguez74_backup@correo.com</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>9261337</v>
+        <v>9974400</v>
       </c>
       <c r="E22" t="n">
-        <v>5191025</v>
+        <v>5893355</v>
       </c>
       <c r="F22" t="n">
-        <v>733</v>
+        <v>343</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Fondo de inversion</t>
+          <t>Fondo de inversion, Pension voluntaria, Cesantias</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1547,39 +1547,39 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>2800959</v>
+        <v>1656820</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>46187.56031574074</v>
+        <v>46186.56031575231</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1090000119</t>
+          <t>1090000132</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Juan Castillo</t>
+          <t>Silvia Perez</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>juan.84@gmail.com</t>
+          <t>silvia.perez55@example.com</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>7049002</v>
+        <v>1866689</v>
       </c>
       <c r="E23" t="n">
-        <v>1122053</v>
+        <v>5423403</v>
       </c>
       <c r="F23" t="n">
-        <v>497</v>
+        <v>685</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Pension obligatoria</t>
+          <t>Pension voluntaria, Seguro de vida, Cesantias</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1597,48 +1597,48 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>4535581</v>
+        <v>1371018</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>46191.56031574074</v>
+        <v>46246.56031575231</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1090000120</t>
+          <t>1090000133</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Diego Sanchez</t>
+          <t>Juan Sanchez</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>diego.sanchez51_backup@correo.com</t>
+          <t>juan.sanchez37_backup@correo.com</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8297927</v>
+        <v>9916258</v>
       </c>
       <c r="E24" t="n">
-        <v>3839880</v>
+        <v>5948983</v>
       </c>
       <c r="F24" t="n">
-        <v>338</v>
+        <v>758</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Fondo de inversion, Pension obligatoria</t>
+          <t>Fondo de inversion, Pension voluntaria, Cesantias</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1647,48 +1647,48 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>4211538</v>
+        <v>3637823</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>46203.56031575231</v>
+        <v>46247.56031575231</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1090000121</t>
+          <t>1090000134</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Roberto Dominguez</t>
+          <t>Maria Ramirez</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>roberto.dominguez18_backup@correo.com</t>
+          <t>maria.ramirez95_backup@correo.com</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>8627814</v>
+        <v>1907355</v>
       </c>
       <c r="E25" t="n">
-        <v>2530938</v>
+        <v>4455291</v>
       </c>
       <c r="F25" t="n">
-        <v>770</v>
+        <v>797</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Pension voluntaria, Pension obligatoria</t>
+          <t>Seguro de vida, Pension voluntaria, Pension obligatoria</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1697,39 +1697,39 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>238829</v>
+        <v>4719054</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="2" t="n">
-        <v>46269.56031575231</v>
+        <v>46203.56031575231</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1090000122</t>
+          <t>1090000135</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Andres Hernandez</t>
+          <t>Sandra Sanchez</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>andres.hernandez79_backup@correo.com</t>
+          <t>sandra.sanchez80_backup@correo.com</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>7852221</v>
+        <v>5483729</v>
       </c>
       <c r="E26" t="n">
-        <v>4043319</v>
+        <v>2162120</v>
       </c>
       <c r="F26" t="n">
-        <v>503</v>
+        <v>414</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1738,57 +1738,57 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Pension voluntaria, Seguro de vida</t>
+          <t>Seguro de vida, Pension voluntaria</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>SUSPENDIDA</t>
+          <t>ACTIVA</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>2447891</v>
+        <v>4157798</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>46192.56031575231</v>
+        <v>46187.56031575231</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1090000123</t>
+          <t>1090000136</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fernando Lopez</t>
+          <t>Carlos Garcia</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>fernando.lopez77_backup@correo.com</t>
+          <t>carlos.garcia6@example.com</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7551769</v>
+        <v>1427689</v>
       </c>
       <c r="E27" t="n">
-        <v>3702630</v>
+        <v>5163608</v>
       </c>
       <c r="F27" t="n">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Seguro de vida, Pension voluntaria</t>
+          <t>Pension obligatoria, Seguro de vida</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1797,39 +1797,39 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>3349132</v>
+        <v>4826466</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>46226.56031575231</v>
+        <v>46201.56031575231</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1090000124</t>
+          <t>1090000137</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Silvia Gutierrez</t>
+          <t>Silvia Castillo</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>silvia.87@outlook.com</t>
+          <t>silvia.68@hotmail.com</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3950157</v>
+        <v>6513863</v>
       </c>
       <c r="E28" t="n">
-        <v>3230906</v>
+        <v>1327904</v>
       </c>
       <c r="F28" t="n">
-        <v>826</v>
+        <v>542</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1838,48 +1838,48 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Pension obligatoria, Cesantias</t>
+          <t>Cesantias</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>ACTIVA</t>
+          <t>SUSPENDIDA</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>3010491</v>
+        <v>4444581</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>46216.56031575231</v>
+        <v>46222.56031575231</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1090000125</t>
+          <t>1090000138</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ana Vargas</t>
+          <t>Jose Rodriguez</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ana.vargas93_backup@correo.com</t>
+          <t>jose.rodriguez6@example.com</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>4762974</v>
+        <v>3673384</v>
       </c>
       <c r="E29" t="n">
-        <v>5360377</v>
+        <v>2263779</v>
       </c>
       <c r="F29" t="n">
-        <v>330</v>
+        <v>683</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1888,98 +1888,98 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Pension obligatoria</t>
+          <t>Fondo de inversion, Pension voluntaria, Seguro de vida</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>SUSPENDIDA</t>
+          <t>ACTIVA</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>1208058</v>
+        <v>2701502</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>46186.56031575231</v>
+        <v>46208.56031575231</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1090000126</t>
+          <t>1090000139</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sandra Ramirez</t>
+          <t>Mariana Lopez</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>sandra.82@outlook.com</t>
+          <t>mariana.lopez73_backup@correo.com</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>5139802</v>
+        <v>568718</v>
       </c>
       <c r="E30" t="n">
-        <v>1606064</v>
+        <v>4962252</v>
       </c>
       <c r="F30" t="n">
-        <v>688</v>
+        <v>735</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Pension voluntaria, Fondo de inversion</t>
+          <t>Cesantias</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>ACTIVA</t>
+          <t>SUSPENDIDA</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>697999</v>
+        <v>4358902</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>46241.56031575231</v>
+        <v>46264.56031575231</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1090000127</t>
+          <t>1090000140</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Miguel Cruz</t>
+          <t>Maria Torres</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>miguel.42@empresa.com.co</t>
+          <t>maria.torres49_backup@correo.com</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2931284</v>
+        <v>9467202</v>
       </c>
       <c r="E31" t="n">
-        <v>2864732</v>
+        <v>3581158</v>
       </c>
       <c r="F31" t="n">
-        <v>463</v>
+        <v>744</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Pension voluntaria</t>
+          <t>Pension obligatoria, Fondo de inversion, Pension voluntaria</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1997,89 +1997,89 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>2382433</v>
+        <v>3733944</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>46263.56031575231</v>
+        <v>46229.56031575231</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1090000128</t>
+          <t>1090000141</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Juan Rodriguez</t>
+          <t>Rosa Dominguez</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>juan.rodriguez62@example.com</t>
+          <t>rosa.dominguez91_backup@correo.com</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>5710501</v>
+        <v>5934832</v>
       </c>
       <c r="E32" t="n">
-        <v>3014887</v>
+        <v>1966269</v>
       </c>
       <c r="F32" t="n">
-        <v>796</v>
+        <v>730</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Fondo de inversion, Pension obligatoria</t>
+          <t>Fondo de inversion, Pension obligatoria, Cesantias</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>SUSPENDIDA</t>
+          <t>ACTIVA</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>2570265</v>
+        <v>3882955</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>46235.56031575231</v>
+        <v>46219.56031575231</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1090000129</t>
+          <t>1090000142</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fernando Dominguez</t>
+          <t>Sandra Rodriguez</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>fernando.dominguez3_backup@correo.com</t>
+          <t>sandra.rodriguez78@example.com</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>9100219</v>
+        <v>1048368</v>
       </c>
       <c r="E33" t="n">
-        <v>4123750</v>
+        <v>5404985</v>
       </c>
       <c r="F33" t="n">
-        <v>422</v>
+        <v>660</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Cesantias</t>
+          <t>Seguro de vida</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2097,89 +2097,89 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>4226540</v>
+        <v>1297602</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>46249.56031575231</v>
+        <v>46213.56031575231</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1090000130</t>
+          <t>1090000143</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Diego Martinez</t>
+          <t>Rosa Ramirez</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>diego.martinez74@example.com</t>
+          <t>rosa.5@yahoo.com</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>7343863</v>
+        <v>2401206</v>
       </c>
       <c r="E34" t="n">
-        <v>4172992</v>
+        <v>5707288</v>
       </c>
       <c r="F34" t="n">
-        <v>380</v>
+        <v>671</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Pension obligatoria, Pension voluntaria, Cesantias</t>
+          <t>Pension voluntaria, Fondo de inversion, Pension obligatoria</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>SUSPENDIDA</t>
+          <t>ACTIVA</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>192832</v>
+        <v>3714425</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>46246.56031575231</v>
+        <v>46214.56031575231</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1090000131</t>
+          <t>1090000144</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Fernando Rodriguez</t>
+          <t>Jose Cruz</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>fernando.rodriguez74_backup@correo.com</t>
+          <t>jose.60@yahoo.com</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>9974400</v>
+        <v>6508620</v>
       </c>
       <c r="E35" t="n">
-        <v>5893355</v>
+        <v>2513257</v>
       </c>
       <c r="F35" t="n">
-        <v>343</v>
+        <v>633</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Fondo de inversion, Pension voluntaria, Cesantias</t>
+          <t>Pension voluntaria</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2197,39 +2197,39 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>1656820</v>
+        <v>3370799</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>46186.56031575231</v>
+        <v>46257.56031575231</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1090000132</t>
+          <t>1090000145</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Silvia Perez</t>
+          <t>Diego Castillo</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>silvia.perez55@example.com</t>
+          <t>diego.castillo35_backup@correo.com</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1866689</v>
+        <v>6349862</v>
       </c>
       <c r="E36" t="n">
-        <v>5423403</v>
+        <v>3386423</v>
       </c>
       <c r="F36" t="n">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2247,48 +2247,48 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>1371018</v>
+        <v>3507895</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>46246.56031575231</v>
+        <v>46263.56031575231</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1090000133</t>
+          <t>1090000146</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Juan Sanchez</t>
+          <t>Silvia Torres</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>juan.sanchez37_backup@correo.com</t>
+          <t>silvia.torres90@example.com</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>9916258</v>
+        <v>5142118</v>
       </c>
       <c r="E37" t="n">
-        <v>5948983</v>
+        <v>2586841</v>
       </c>
       <c r="F37" t="n">
-        <v>758</v>
+        <v>552</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Fondo de inversion, Pension voluntaria, Cesantias</t>
+          <t>Seguro de vida, Pension voluntaria, Pension obligatoria</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2297,89 +2297,89 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>3637823</v>
+        <v>1664523</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>46247.56031575231</v>
+        <v>46271.56031575231</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1090000134</t>
+          <t>1090000147</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Maria Ramirez</t>
+          <t>Jose Torres</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>maria.ramirez95_backup@correo.com</t>
+          <t>jose.torres31_backup@correo.com</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1907355</v>
+        <v>4939729</v>
       </c>
       <c r="E38" t="n">
-        <v>4455291</v>
+        <v>4779479</v>
       </c>
       <c r="F38" t="n">
-        <v>797</v>
+        <v>496</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Seguro de vida, Pension voluntaria, Pension obligatoria</t>
+          <t>Pension voluntaria, Seguro de vida</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>ACTIVA</t>
+          <t>SUSPENDIDA</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>4719054</v>
+        <v>1380956</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>46203.56031575231</v>
+        <v>46251.56031575231</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1090000135</t>
+          <t>1090000148</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Sandra Sanchez</t>
+          <t>Carlos Rodriguez</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>sandra.sanchez80_backup@correo.com</t>
+          <t>carlos.rodriguez51_backup@correo.com</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>5483729</v>
+        <v>9210158</v>
       </c>
       <c r="E39" t="n">
-        <v>2162120</v>
+        <v>2493868</v>
       </c>
       <c r="F39" t="n">
-        <v>414</v>
+        <v>527</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2388,57 +2388,57 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Seguro de vida, Pension voluntaria</t>
+          <t>Pension voluntaria, Pension obligatoria</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>ACTIVA</t>
+          <t>SUSPENDIDA</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>4157798</v>
+        <v>4694707</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>46187.56031575231</v>
+        <v>46266.56031575231</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1090000136</t>
+          <t>1090000149</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Carlos Garcia</t>
+          <t>Miguel Vargas</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>carlos.garcia6@example.com</t>
+          <t>miguel.vargas20@example.com</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1427689</v>
+        <v>3602837</v>
       </c>
       <c r="E40" t="n">
-        <v>5163608</v>
+        <v>3659094</v>
       </c>
       <c r="F40" t="n">
-        <v>765</v>
+        <v>652</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Pension obligatoria, Seguro de vida</t>
+          <t>Seguro de vida, Pension voluntaria</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2447,662 +2447,12 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>4826466</v>
+        <v>298351</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>46201.56031575231</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>1090000137</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Silvia Castillo</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>silvia.68@hotmail.com</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>6513863</v>
-      </c>
-      <c r="E41" t="n">
-        <v>1327904</v>
-      </c>
-      <c r="F41" t="n">
-        <v>542</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>BAJO</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Cesantias</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>SUSPENDIDA</t>
-        </is>
-      </c>
-      <c r="J41" t="n">
-        <v>4444581</v>
-      </c>
-      <c r="K41" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" s="2" t="n">
-        <v>46222.56031575231</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>1090000138</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Jose Rodriguez</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>jose.rodriguez6@example.com</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>3673384</v>
-      </c>
-      <c r="E42" t="n">
-        <v>2263779</v>
-      </c>
-      <c r="F42" t="n">
-        <v>683</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>BAJO</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Fondo de inversion, Pension voluntaria, Seguro de vida</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>ACTIVA</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>2701502</v>
-      </c>
-      <c r="K42" t="n">
-        <v>0</v>
-      </c>
-      <c r="L42" s="2" t="n">
-        <v>46208.56031575231</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>1090000139</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Mariana Lopez</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>mariana.lopez73_backup@correo.com</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>568718</v>
-      </c>
-      <c r="E43" t="n">
-        <v>4962252</v>
-      </c>
-      <c r="F43" t="n">
-        <v>735</v>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>ALTO</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Cesantias</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>SUSPENDIDA</t>
-        </is>
-      </c>
-      <c r="J43" t="n">
-        <v>4358902</v>
-      </c>
-      <c r="K43" t="n">
-        <v>0</v>
-      </c>
-      <c r="L43" s="2" t="n">
-        <v>46264.56031575231</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>1090000140</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Maria Torres</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>maria.torres49_backup@correo.com</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>9467202</v>
-      </c>
-      <c r="E44" t="n">
-        <v>3581158</v>
-      </c>
-      <c r="F44" t="n">
-        <v>744</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>MEDIO</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Pension obligatoria, Fondo de inversion, Pension voluntaria</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>ACTIVA</t>
-        </is>
-      </c>
-      <c r="J44" t="n">
-        <v>3733944</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" s="2" t="n">
-        <v>46229.56031575231</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>1090000141</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Rosa Dominguez</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>rosa.dominguez91_backup@correo.com</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>5934832</v>
-      </c>
-      <c r="E45" t="n">
-        <v>1966269</v>
-      </c>
-      <c r="F45" t="n">
-        <v>730</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>ALTO</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Fondo de inversion, Pension obligatoria, Cesantias</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>ACTIVA</t>
-        </is>
-      </c>
-      <c r="J45" t="n">
-        <v>3882955</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" s="2" t="n">
-        <v>46219.56031575231</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>1090000142</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Sandra Rodriguez</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>sandra.rodriguez78@example.com</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>1048368</v>
-      </c>
-      <c r="E46" t="n">
-        <v>5404985</v>
-      </c>
-      <c r="F46" t="n">
-        <v>660</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>BAJO</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Seguro de vida</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>ACTIVA</t>
-        </is>
-      </c>
-      <c r="J46" t="n">
-        <v>1297602</v>
-      </c>
-      <c r="K46" t="n">
-        <v>0</v>
-      </c>
-      <c r="L46" s="2" t="n">
-        <v>46213.56031575231</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>1090000143</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Rosa Ramirez</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>rosa.5@yahoo.com</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>2401206</v>
-      </c>
-      <c r="E47" t="n">
-        <v>5707288</v>
-      </c>
-      <c r="F47" t="n">
-        <v>671</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>BAJO</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Pension voluntaria, Fondo de inversion, Pension obligatoria</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>ACTIVA</t>
-        </is>
-      </c>
-      <c r="J47" t="n">
-        <v>3714425</v>
-      </c>
-      <c r="K47" t="n">
-        <v>0</v>
-      </c>
-      <c r="L47" s="2" t="n">
-        <v>46214.56031575231</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>1090000144</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Jose Cruz</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>jose.60@yahoo.com</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>6508620</v>
-      </c>
-      <c r="E48" t="n">
-        <v>2513257</v>
-      </c>
-      <c r="F48" t="n">
-        <v>633</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>BAJO</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Pension voluntaria</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>ACTIVA</t>
-        </is>
-      </c>
-      <c r="J48" t="n">
-        <v>3370799</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0</v>
-      </c>
-      <c r="L48" s="2" t="n">
-        <v>46257.56031575231</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>1090000145</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Diego Castillo</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>diego.castillo35_backup@correo.com</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
-        <v>6349862</v>
-      </c>
-      <c r="E49" t="n">
-        <v>3386423</v>
-      </c>
-      <c r="F49" t="n">
-        <v>692</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>BAJO</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Pension voluntaria, Seguro de vida, Cesantias</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>ACTIVA</t>
-        </is>
-      </c>
-      <c r="J49" t="n">
-        <v>3507895</v>
-      </c>
-      <c r="K49" t="n">
-        <v>0</v>
-      </c>
-      <c r="L49" s="2" t="n">
-        <v>46263.56031575231</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>1090000146</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Silvia Torres</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>silvia.torres90@example.com</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>5142118</v>
-      </c>
-      <c r="E50" t="n">
-        <v>2586841</v>
-      </c>
-      <c r="F50" t="n">
-        <v>552</v>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>ALTO</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Seguro de vida, Pension voluntaria, Pension obligatoria</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>ACTIVA</t>
-        </is>
-      </c>
-      <c r="J50" t="n">
-        <v>1664523</v>
-      </c>
-      <c r="K50" t="n">
-        <v>0</v>
-      </c>
-      <c r="L50" s="2" t="n">
-        <v>46271.56031575231</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>1090000147</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Jose Torres</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>jose.torres31_backup@correo.com</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>4939729</v>
-      </c>
-      <c r="E51" t="n">
-        <v>4779479</v>
-      </c>
-      <c r="F51" t="n">
-        <v>496</v>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>MEDIO</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Pension voluntaria, Seguro de vida</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>SUSPENDIDA</t>
-        </is>
-      </c>
-      <c r="J51" t="n">
-        <v>1380956</v>
-      </c>
-      <c r="K51" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" s="2" t="n">
-        <v>46251.56031575231</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>1090000148</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Carlos Rodriguez</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>carlos.rodriguez51_backup@correo.com</t>
-        </is>
-      </c>
-      <c r="D52" t="n">
-        <v>9210158</v>
-      </c>
-      <c r="E52" t="n">
-        <v>2493868</v>
-      </c>
-      <c r="F52" t="n">
-        <v>527</v>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>BAJO</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Pension voluntaria, Pension obligatoria</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>SUSPENDIDA</t>
-        </is>
-      </c>
-      <c r="J52" t="n">
-        <v>4694707</v>
-      </c>
-      <c r="K52" t="n">
-        <v>15</v>
-      </c>
-      <c r="L52" s="2" t="n">
-        <v>46266.56031575231</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>1090000149</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Miguel Vargas</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>miguel.vargas20@example.com</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>3602837</v>
-      </c>
-      <c r="E53" t="n">
-        <v>3659094</v>
-      </c>
-      <c r="F53" t="n">
-        <v>652</v>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>MEDIO</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Seguro de vida, Pension voluntaria</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>SUSPENDIDA</t>
-        </is>
-      </c>
-      <c r="J53" t="n">
-        <v>298351</v>
-      </c>
-      <c r="K53" t="n">
-        <v>0</v>
-      </c>
-      <c r="L53" s="2" t="n">
         <v>46262.56031575231</v>
       </c>
     </row>

</xml_diff>